<commit_message>
Resolve Mission Brief asset ambiguity: EX001 reused
DECISIONS.md #013 — EX001 (Mission Control) is repurposed from its
original Exercise/Segment-8 categorization to the in-scope Mission
Brief scene. EX002 (Apex Dossier) stays out of scope. Asset_Register
updated (category, description, notes); Scene Bible Scene 6 and
§3.3 updated to reflect the resolution.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Asset_Register_v1.0.xlsx
+++ b/docs/Asset_Register_v1.0.xlsx
@@ -508,7 +508,6 @@
           <t>OpenAI Images</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -588,13 +587,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>OpenAI Images</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -627,13 +624,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>OpenAI Images</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -666,13 +661,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>OpenAI Images</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -705,13 +698,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>OpenAI Images</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -744,13 +735,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>OpenAI Images</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -783,13 +772,11 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>OpenAI Images</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -822,13 +809,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>OpenAI Images</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -861,13 +846,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>OpenAI Images</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -900,13 +883,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>OpenAI Images</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -939,13 +920,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>HTML/SVG</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -978,13 +957,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>OpenAI Images</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1017,13 +994,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>SVG/HTML</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1056,13 +1031,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>OpenAI Images</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1095,13 +1068,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>SVG</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1134,13 +1105,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>OpenAI Images</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1173,13 +1142,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>OpenAI Images</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1212,13 +1179,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>OpenAI Images</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1251,13 +1216,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>OpenAI Images</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1290,13 +1253,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>OpenAI Images</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1329,13 +1290,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>OpenAI Images</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1345,7 +1304,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Exercise</t>
+          <t>Mission Brief</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1355,7 +1314,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Apex briefing</t>
+          <t>Post-Mission-Board wrap scene, before Debrief (reused from original Exercise/Apex-briefing concept)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1368,13 +1327,16 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>HTML/SVG</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Repurposed from Segment 8 (Exercise, out of scope) per 2026-08-06 decision — see DECISIONS.md #013, Scene Bible Scene 6</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1407,13 +1369,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>HTML/SVG</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1446,13 +1406,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>HTML</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1485,13 +1443,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>OpenAI Images</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1524,13 +1480,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>OpenAI Images</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1563,13 +1517,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>OpenAI Images</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1602,13 +1554,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>SVG</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1641,13 +1591,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>SVG</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1680,13 +1628,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>HTML/CSS</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1729,7 +1675,6 @@
           <t>CC0</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1772,7 +1717,6 @@
           <t>CC0</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Resolve all remaining Milestone 1 open items
DECISIONS.md #015-#019:
- Easter Egg Wall assets registered as EE001-EE004 (Cold Open,
  Medium priority, HTML/CSS-animated text rather than video)
- Minimum hardware baseline confirmed (dual-core ~2.0GHz+, 8GB RAM,
  integrated graphics, 1280x800 min., evergreen browser)
- Release size budget confirmed at <=150MB
- Audio confirmed required-to-ship, playback failure stays
  non-blocking per NFR-6
- Cold Open / Operations Centre split confirmed as interpreted in
  Scene_Bible.md Sec 2.1

Updated SRS (NFR-4/5, Sec 8), Architecture (Sec 8, Sec 11),
Scene Bible (Sec 2.1, Sec 3.1), Asset_Register (+4 rows), TODO.md.
No open items remain from Milestone 1's spec review.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Asset_Register_v1.0.xlsx
+++ b/docs/Asset_Register_v1.0.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1718,6 +1718,174 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>EE001</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Cold Open</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Python Monitor</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Easter Egg Wall — looping Python interpreter session, buried signature line (Lt Col Dheeraj Bharti, JSACW) legible only on close inspection</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>To Generate</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>HTML/CSS</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Non-video, CSS-animated monospace text scroll per Architecture.md C-12; DECISIONS.md #015</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>EE002</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Cold Open</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Networking Monitor</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Easter Egg Wall — ip addr / subnet math scratch notes, background packet capture scroll</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>To Generate</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>HTML/CSS</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Non-video, CSS-animated monospace text scroll; DECISIONS.md #015</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>EE003</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Cold Open</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>PowerShell Monitor</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Easter Egg Wall — AD enumeration commands, Windows fundamentals references scrolling past</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>To Generate</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>HTML/CSS</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Non-video, CSS-animated monospace text scroll; DECISIONS.md #015</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>EE004</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Cold Open</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Bash Monitor</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Easter Egg Wall — shell scripting loop, permissions/chmod examples</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>To Generate</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>HTML/CSS</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Non-video, CSS-animated monospace text scroll; DECISIONS.md #015</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Milestone 2: prompt library + first 4 concept-art assets
- Build prompts/ library (style_lock.md + assets.json, 22 assets)
- Explore Gemini API (Imagen) generation — DECISIONS.md #020;
  blocked by 0 image-model quota on free tier (#021), script kept
  for future use once billing is enabled
- Explore Unsplash stock photo + CSS/SVG overlay hybrid — DECISIONS.md
  #021/#022; API keys configured, no script built before the plan
  changed
- Settle on manual ChatGPT generation for all 22 assets (#023):
  4 generated and placed (A001, A002, B003, SB001 -> assets/images/
  as .webp), remaining 18 handed off as prompts/remaining_18_prompts.md
  (zipped) for manual generation and hand-back
- Add .env.example (UNSPLASH_*, GEMINI_API_KEY, OPENAI_API_KEY,
  FIRECRAWL_API_KEY), gitignore /images/ staging folder
- Update Asset_Register_v1.0.xlsx Source column and TODO.md throughout

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Asset_Register_v1.0.xlsx
+++ b/docs/Asset_Register_v1.0.xlsx
@@ -490,7 +490,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>To Generate</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -505,7 +505,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>OpenAI Images</t>
+          <t>ChatGPT (manual)</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Generated 2026-08-06 per DECISIONS.md #022 prompts; converted to .webp, pending final review</t>
         </is>
       </c>
     </row>
@@ -547,12 +552,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>OpenAI Images</t>
+          <t>ChatGPT (manual)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Approved concept</t>
+          <t>Generated 2026-08-06 per DECISIONS.md #022 prompts; converted to .webp, pending final review</t>
         </is>
       </c>
     </row>
@@ -589,7 +594,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>OpenAI Images</t>
+          <t>ChatGPT (manual)</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
         </is>
       </c>
     </row>
@@ -626,7 +636,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>OpenAI Images</t>
+          <t>ChatGPT (manual)</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
         </is>
       </c>
     </row>
@@ -653,7 +668,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>To Generate</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -663,7 +678,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>OpenAI Images</t>
+          <t>ChatGPT (manual)</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Generated 2026-08-06 per DECISIONS.md #022 prompts; converted to .webp, pending final review</t>
         </is>
       </c>
     </row>
@@ -700,7 +720,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>OpenAI Images</t>
+          <t>ChatGPT (manual)</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
         </is>
       </c>
     </row>
@@ -737,7 +762,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>OpenAI Images</t>
+          <t>ChatGPT (manual)</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
         </is>
       </c>
     </row>
@@ -774,7 +804,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>OpenAI Images</t>
+          <t>ChatGPT (manual)</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
         </is>
       </c>
     </row>
@@ -811,7 +846,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>OpenAI Images</t>
+          <t>ChatGPT (manual)</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
         </is>
       </c>
     </row>
@@ -848,7 +888,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>OpenAI Images</t>
+          <t>ChatGPT (manual)</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
         </is>
       </c>
     </row>
@@ -885,7 +930,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>OpenAI Images</t>
+          <t>ChatGPT (manual)</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
         </is>
       </c>
     </row>
@@ -959,7 +1009,12 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>OpenAI Images</t>
+          <t>ChatGPT (manual)</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1088,12 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>OpenAI Images</t>
+          <t>ChatGPT (manual)</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1167,12 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>OpenAI Images</t>
+          <t>ChatGPT (manual)</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1209,12 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>OpenAI Images</t>
+          <t>ChatGPT (manual)</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1251,12 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>OpenAI Images</t>
+          <t>ChatGPT (manual)</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
         </is>
       </c>
     </row>
@@ -1208,7 +1283,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>To Generate</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1218,7 +1293,12 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>OpenAI Images</t>
+          <t>ChatGPT (manual)</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Generated 2026-08-06 per DECISIONS.md #022 prompts; converted to .webp, pending final review</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1335,12 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>OpenAI Images</t>
+          <t>ChatGPT (manual)</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
         </is>
       </c>
     </row>
@@ -1292,7 +1377,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>OpenAI Images</t>
+          <t>ChatGPT (manual)</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
         </is>
       </c>
     </row>
@@ -1445,7 +1535,12 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>OpenAI Images</t>
+          <t>ChatGPT (manual)</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
         </is>
       </c>
     </row>
@@ -1482,7 +1577,12 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>OpenAI Images</t>
+          <t>ChatGPT (manual)</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
         </is>
       </c>
     </row>
@@ -1519,7 +1619,12 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>OpenAI Images</t>
+          <t>ChatGPT (manual)</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Source AU001/AU002 audio loops (CC0, Freesound)
- rain.ogg: "Rain from Indoors - Perfect loop" by samesamesame,
  freesound.org/s/242889, CC0, 48s
- ops.ogg: "AMBTech_Server Room Noise 01_KVV_FREE" by KVV_Audio,
  freesound.org/s/715475, CC0, 1:42
- Converted MP3 -> OGG (vorbis) via ffmpeg, placed in assets/audio/
- DECISIONS.md #024: switched from the initially-approved Pixabay
  candidates after their download flow proved unscriptable
  (Cloudflare-protected SPA); Freesound's CDN serves preview files
  directly and its license is genuinely CC0, matching the Asset
  Register's stated requirement more precisely than Pixabay's
  similar-but-distinct Content License
- Asset_Register_v1.0.xlsx: AU001/AU002 marked Ready with attribution

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Asset_Register_v1.0.xlsx
+++ b/docs/Asset_Register_v1.0.xlsx
@@ -1762,7 +1762,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>To Source</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1778,6 +1778,11 @@
       <c r="H33" t="inlineStr">
         <is>
           <t>CC0</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Rain from Indoors - Perfect loop by samesamesame, freesound.org/s/242889, CC0, 48s</t>
         </is>
       </c>
     </row>
@@ -1804,7 +1809,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>To Source</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1820,6 +1825,11 @@
       <c r="H34" t="inlineStr">
         <is>
           <t>CC0</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>AMBTech_Server Room Noise 01 by KVV_Audio, freesound.org/s/715475, CC0, 1:42</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Process 13 more generated concept-art assets
B001, B002, C001, C004, C005, D001, D003, F001, FC001, GA001, GD001,
SG001, TC001 converted to .webp and placed in assets/images/.
17/22 image assets now done; 5 remaining (ST001, GP001, DB001, EN001,
EN002). Asset_Register_v1.0.xlsx and prompts/assets.json status
updated accordingly.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Asset_Register_v1.0.xlsx
+++ b/docs/Asset_Register_v1.0.xlsx
@@ -584,7 +584,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>To Generate</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -599,7 +599,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
+          <t>Generated 2026-08-06 per DECISIONS.md #023 prompts; converted to .webp, pending final review</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>To Generate</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -641,7 +641,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
+          <t>Generated 2026-08-06 per DECISIONS.md #023 prompts; converted to .webp, pending final review</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>To Generate</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
+          <t>Generated 2026-08-06 per DECISIONS.md #023 prompts; converted to .webp, pending final review</t>
         </is>
       </c>
     </row>
@@ -752,7 +752,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>To Generate</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -767,7 +767,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
+          <t>Generated 2026-08-06 per DECISIONS.md #023 prompts; converted to .webp, pending final review</t>
         </is>
       </c>
     </row>
@@ -794,7 +794,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>To Generate</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -809,7 +809,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
+          <t>Generated 2026-08-06 per DECISIONS.md #023 prompts; converted to .webp, pending final review</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>To Generate</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -851,7 +851,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
+          <t>Generated 2026-08-06 per DECISIONS.md #023 prompts; converted to .webp, pending final review</t>
         </is>
       </c>
     </row>
@@ -878,7 +878,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>To Generate</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -893,7 +893,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
+          <t>Generated 2026-08-06 per DECISIONS.md #023 prompts; converted to .webp, pending final review</t>
         </is>
       </c>
     </row>
@@ -920,7 +920,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>To Generate</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
+          <t>Generated 2026-08-06 per DECISIONS.md #023 prompts; converted to .webp, pending final review</t>
         </is>
       </c>
     </row>
@@ -999,7 +999,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>To Generate</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1014,7 +1014,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
+          <t>Generated 2026-08-06 per DECISIONS.md #023 prompts; converted to .webp, pending final review</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>To Generate</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
+          <t>Generated 2026-08-06 per DECISIONS.md #023 prompts; converted to .webp, pending final review</t>
         </is>
       </c>
     </row>
@@ -1157,7 +1157,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>To Generate</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1172,7 +1172,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
+          <t>Generated 2026-08-06 per DECISIONS.md #023 prompts; converted to .webp, pending final review</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>To Generate</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
+          <t>Generated 2026-08-06 per DECISIONS.md #023 prompts; converted to .webp, pending final review</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>To Generate</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
+          <t>Generated 2026-08-06 per DECISIONS.md #023 prompts; converted to .webp, pending final review</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Process ST001 concept-art asset
18/22 image assets now done; 4 remaining (GP001, DB001, EN001, EN002).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Asset_Register_v1.0.xlsx
+++ b/docs/Asset_Register_v1.0.xlsx
@@ -1325,7 +1325,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>To Generate</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
+          <t>Generated 2026-08-06 per DECISIONS.md #023 prompts; converted to .webp, pending final review</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Process DB001, GP001, EN002 concept-art assets
21/22 image assets now done; only EN001 (Lane Return) remains.
EN002 source file was named EN002_png.png rather than the expected
EN002_hack_meth_reveal.png -- mapped by asset ID rather than filename.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Asset_Register_v1.0.xlsx
+++ b/docs/Asset_Register_v1.0.xlsx
@@ -1367,7 +1367,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>To Generate</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
+          <t>Generated 2026-08-06 per DECISIONS.md #023 prompts; converted to .webp, pending final review</t>
         </is>
       </c>
     </row>
@@ -1525,7 +1525,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>To Generate</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
+          <t>Generated 2026-08-06 per DECISIONS.md #023 prompts; converted to .webp, pending final review</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>To Generate</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1624,7 +1624,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
+          <t>Generated 2026-08-06 per DECISIONS.md #023 prompts; converted to .webp, pending final review</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Process EN001 -- Milestone 2 image generation complete (22/22)
All 22 registered image assets generated and placed in assets/images/
as .webp (6.8MB total, well under the 150MB budget). Audio (2/2) was
already done. Remaining Asset Register "To Generate" rows are
HTML/SVG/CSS build-time components for Milestone 3, not images.
Milestone 2's asset-generation scope is complete pending final
review of the Draft-status images.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Asset_Register_v1.0.xlsx
+++ b/docs/Asset_Register_v1.0.xlsx
@@ -1567,7 +1567,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>To Generate</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Prompt in prompts/remaining_18_prompts.md, handed off 2026-08-06 (DECISIONS.md #023)</t>
+          <t>Generated 2026-08-06 per DECISIONS.md #023 prompts; converted to .webp, pending final review</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate and place EN002, DB001 -- 22/22 images now placed
EN002: corrected signage confirmed ("HACK METH"), passes review clean.

DB001: real Mission Debrief content generated at last (previous file
was wrong room entirely). Content/checklist matches the real 9-room
scope. Flagged, not clean: the "Next Destination" panel reads both
"HACK METH" and "RED TEAM OPS AWAITS" in the same image (self-
contradicting, violates DECISIONS.md #012), and bakes in YES/NOT YET
buttons as static art rather than leaving them for real HTML controls.

All 22 assets are now placed; 4 still have open decisions pending
before any can move from Draft to Ready (see TODO.md).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Asset_Register_v1.0.xlsx
+++ b/docs/Asset_Register_v1.0.xlsx
@@ -1525,7 +1525,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>To Generate</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>REVERTED 2026-08-06: file previously registered here contained "Dark Web Investigations Room" content, not Mission Debrief, and does not match any Version-1 room. Moved to assets/images/_rejected/. Needs regeneration.</t>
+          <t>Generated 2026-08-06. Content/checklist accurate to 9-room scope. ISSUE: bottom panel reads both HACK METH and RED TEAM OPS AWAITS in the same image, self-contradicting and violating DECISIONS.md #012 on the latter. Also bakes in YES/NOT YET buttons as static art -- must be real HTML controls at build time, not pixels.</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>To Generate</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1624,7 +1624,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>REVERTED 2026-08-06: generated image rendered "RED TEAM OPS" signage, violating DECISIONS.md #012 (HACK METH prevails). Moved to assets/images/_rejected/. Needs regeneration with corrected signage text.</t>
+          <t>Regenerated 2026-08-06 with corrected HACK METH signage per DECISIONS.md #012. Passes review.</t>
         </is>
       </c>
     </row>

</xml_diff>